<commit_message>
자료실: A.i 컨텐츠 결제 안내서(한/영) + 관리자용 사용설명서 10장 «AI 컨텐츠 결제» / Library: A.i content payment guide (KO/EN) + admin guide ch.10
- 대리점 자료실·관리자 자료실 맨 위에 «🤖 A.i 컨텐츠 결제 안내서»(A4 4쪽, 한/영 · 열기·저장·카톡 링크)
  /library/agency/ai-pay-guide-kr|en.pdf — 같은 파일을 두 자료실이 연다
- 사장님 PDF 는 로그인 사진에 실제 대리점 아이디가 있어 같은 구성으로 다시 만듦
  (시연 계정 testagency 캡처 · sample01 · 「2쪽 표」→「끝쪽 표」) — 원본 docs/자료실_원본/AI컨텐츠_결제안내/
- 관리자용 사용설명서 10장 «AI 컨텐츠 결제(대리점)» 6단계 + FAQ 3 → 10장 45단계, PDF/PPTX/XLSX 한/영 재생성
  1~9장 그림은 배포된 PPTX 에서 단계 제목으로 대조해 되살림(restore_images.py) — 글·그림 어긋남 방지
- 두 빌드가 쓰는 크로미움 띄우기·글꼴 심기를 docs/자료실_원본/_공용/pdf-helpers.mjs 로 모음(옛 chromium-1194 경로 하드코딩 제거)
- 작업기록·INDEX·CLAUDE.md 2장 함정 1줄(사람이 준 자료 속 실제 아이디)

Add the A.i content payment guide (A4, 4 pages, KO/EN) to the agency and admin libraries,
and add chapter 10 (A.i content payment) to the admin user guide (PDF/PPTX/XLSX, KO/EN).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015hjUTfinHmjG25a7d4k1UA
</commit_message>
<xml_diff>
--- a/cloudflare-deploy/public/library/admin/admin-en.xlsx
+++ b/cloudflare-deploy/public/library/admin/admin-en.xlsx
@@ -1111,6 +1111,156 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1241</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2962275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1260</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4724400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1288</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3895725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1312</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2181225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1327</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3800475"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1350</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="1200150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1413,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2796,6 +2946,213 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>10-1</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Agency login · open the menu</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>• An agency logs in at mangoi.ai/admin/login with its agency ID and gets the agency screen.
+• ④ Left menu Settlement &amp; stats › 🤖 A.i content payment. This menu appears only for agency accounts (not for HQ or branch accounts).
+• HQ uses Finance › 🏢 AI Usage Fee (A.i Learning Fee Management) to see each academy’s headcount and estimated invoice, set custom rates, and turn auto-billing on or off. There is no pay button there.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>10-2</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Load the student list</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>• Check the due date at the top (last day of this month · D-days left). The payment is for next month.
+• Counters: Signed up for A.i (to be paid) · Not signed up · Video class (included) — video-class students get A.i with their tuition and are not paid here.
+• ⑤ Load my students and choose only loads the list. Nothing is paid at this point.
+• If HQ has not turned on auto-billing yet, the agency only sees «Head office has not opened A.i content payment yet (test period)» — it is not broken.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>10-3</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Choose next month’s students</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>• ⑥ Only students checked under Paying for A.i content are paid. Unchecking a student who left removes them before payment.
+• Search by name or ID; Unselect all shown / Select all shown changes many at once (it asks how many first).
+• The server recalculates the amount every time a check changes.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>10-4</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Not signed up · video-class students</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>• ⑦ Checking a student under Not signed up adds them to the payment.
+• 📹 Video-class students are folded away. A.i is included in their tuition, so they are not chosen — check one only if the classification is wrong.
+• Students the academy changed get a «✔ confirmed by academy» tag, and automatic classification no longer changes them.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>10-5</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Check the amount · pay by card</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>• ⑧ Check the number of students and the total, then ⑨ Pay OOO KRW → confirm → pay in the Toss card window.
+• Price per student per month: 20 or fewer 7,500 · 21–50 6,500 · 51–70 5,500 · 71 or more 4,500 KRW. No minimum charge (since 2026-10-26).
+• The total never goes down as students are added (e.g. 21–23 students = 150,000 KRW). The server recalculates the amount at the moment of payment — the screen number is for display. Academies with an HQ custom rate pay that rate × students.
+• The demo account (testagency) does not open the payment window (sample data).</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>10-6</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Check the payment · extra payment</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>• ⑩ A ✅ under Past payments means paid. After paying, «Paid» appears and paid students are pinned at the top.
+• To add students in the same month, check them below and press Pay extra — only the added students are charged.
+• Students already paid for cannot be removed or changed on the screen. HQ handles refunds.
+• If an earlier month is unpaid, a «⚠️ Unpaid A.i content invoice(s)» button appears at the top.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2807,7 +3164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1209"/>
+  <dimension ref="A1:A1350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3083,6 +3440,48 @@
       <c r="A1209" s="3" t="inlineStr">
         <is>
           <t>9-2  Daily handover</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="3" t="inlineStr">
+        <is>
+          <t>10-1  Agency login · open the menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="3" t="inlineStr">
+        <is>
+          <t>10-2  Load the student list</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="3" t="inlineStr">
+        <is>
+          <t>10-3  Choose next month’s students</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="3" t="inlineStr">
+        <is>
+          <t>10-4  Not signed up · video-class students</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="3" t="inlineStr">
+        <is>
+          <t>10-5  Check the amount · pay by card</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="3" t="inlineStr">
+        <is>
+          <t>10-6  Check the payment · extra payment</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3213,6 +3612,42 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>An agency says it has no «A.i content payment» menu</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Check that they logged in with the agency ID. The menu appears only for agency accounts (not branch or HQ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>An agency sees «Head office has not opened A.i content payment yet»</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>It is not broken. It shows until HQ presses «Turn ON» for auto-billing in Finance › 🏢 AI Usage Fee (test period).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>An agency wants to remove a student they already paid for</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>It cannot be done on the agency screen. HQ handles refunds.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
자료실: A.i 컨텐츠 결제 안내서(한/영) + 관리자용 사용설명서 10장 «AI 컨텐츠 결제» / Library: A.i content payment guide (KO/EN) + admin guide ch.10 (#1847)
- 대리점 자료실·관리자 자료실 맨 위에 «🤖 A.i 컨텐츠 결제 안내서»(A4 4쪽, 한/영 · 열기·저장·카톡 링크)
  /library/agency/ai-pay-guide-kr|en.pdf — 같은 파일을 두 자료실이 연다
- 사장님 PDF 는 로그인 사진에 실제 대리점 아이디가 있어 같은 구성으로 다시 만듦
  (시연 계정 testagency 캡처 · sample01 · 「2쪽 표」→「끝쪽 표」) — 원본 docs/자료실_원본/AI컨텐츠_결제안내/
- 관리자용 사용설명서 10장 «AI 컨텐츠 결제(대리점)» 6단계 + FAQ 3 → 10장 45단계, PDF/PPTX/XLSX 한/영 재생성
  1~9장 그림은 배포된 PPTX 에서 단계 제목으로 대조해 되살림(restore_images.py) — 글·그림 어긋남 방지
- 두 빌드가 쓰는 크로미움 띄우기·글꼴 심기를 docs/자료실_원본/_공용/pdf-helpers.mjs 로 모음(옛 chromium-1194 경로 하드코딩 제거)
- 작업기록·INDEX·CLAUDE.md 2장 함정 1줄(사람이 준 자료 속 실제 아이디)

Add the A.i content payment guide (A4, 4 pages, KO/EN) to the agency and admin libraries,
and add chapter 10 (A.i content payment) to the admin user guide (PDF/PPTX/XLSX, KO/EN).


Claude-Session: https://claude.ai/code/session_015hjUTfinHmjG25a7d4k1UA

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cloudflare-deploy/public/library/admin/admin-en.xlsx
+++ b/cloudflare-deploy/public/library/admin/admin-en.xlsx
@@ -1111,6 +1111,156 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1241</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2962275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1260</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4724400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1288</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3895725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1312</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2181225"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1327</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3800475"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1350</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="1200150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1413,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2796,6 +2946,213 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>10-1</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Agency login · open the menu</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>• An agency logs in at mangoi.ai/admin/login with its agency ID and gets the agency screen.
+• ④ Left menu Settlement &amp; stats › 🤖 A.i content payment. This menu appears only for agency accounts (not for HQ or branch accounts).
+• HQ uses Finance › 🏢 AI Usage Fee (A.i Learning Fee Management) to see each academy’s headcount and estimated invoice, set custom rates, and turn auto-billing on or off. There is no pay button there.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>10-2</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Load the student list</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>• Check the due date at the top (last day of this month · D-days left). The payment is for next month.
+• Counters: Signed up for A.i (to be paid) · Not signed up · Video class (included) — video-class students get A.i with their tuition and are not paid here.
+• ⑤ Load my students and choose only loads the list. Nothing is paid at this point.
+• If HQ has not turned on auto-billing yet, the agency only sees «Head office has not opened A.i content payment yet (test period)» — it is not broken.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>10-3</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Choose next month’s students</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>• ⑥ Only students checked under Paying for A.i content are paid. Unchecking a student who left removes them before payment.
+• Search by name or ID; Unselect all shown / Select all shown changes many at once (it asks how many first).
+• The server recalculates the amount every time a check changes.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>10-4</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Not signed up · video-class students</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>• ⑦ Checking a student under Not signed up adds them to the payment.
+• 📹 Video-class students are folded away. A.i is included in their tuition, so they are not chosen — check one only if the classification is wrong.
+• Students the academy changed get a «✔ confirmed by academy» tag, and automatic classification no longer changes them.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>10-5</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Check the amount · pay by card</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>• ⑧ Check the number of students and the total, then ⑨ Pay OOO KRW → confirm → pay in the Toss card window.
+• Price per student per month: 20 or fewer 7,500 · 21–50 6,500 · 51–70 5,500 · 71 or more 4,500 KRW. No minimum charge (since 2026-10-26).
+• The total never goes down as students are added (e.g. 21–23 students = 150,000 KRW). The server recalculates the amount at the moment of payment — the screen number is for display. Academies with an HQ custom rate pay that rate × students.
+• The demo account (testagency) does not open the payment window (sample data).</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>A.i content payment (agencies)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>10-6</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Check the payment · extra payment</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>• ⑩ A ✅ under Past payments means paid. After paying, «Paid» appears and paid students are pinned at the top.
+• To add students in the same month, check them below and press Pay extra — only the added students are charged.
+• Students already paid for cannot be removed or changed on the screen. HQ handles refunds.
+• If an earlier month is unpaid, a «⚠️ Unpaid A.i content invoice(s)» button appears at the top.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Screens!10-6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2807,7 +3164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1209"/>
+  <dimension ref="A1:A1350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3083,6 +3440,48 @@
       <c r="A1209" s="3" t="inlineStr">
         <is>
           <t>9-2  Daily handover</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="3" t="inlineStr">
+        <is>
+          <t>10-1  Agency login · open the menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="3" t="inlineStr">
+        <is>
+          <t>10-2  Load the student list</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="3" t="inlineStr">
+        <is>
+          <t>10-3  Choose next month’s students</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="3" t="inlineStr">
+        <is>
+          <t>10-4  Not signed up · video-class students</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="3" t="inlineStr">
+        <is>
+          <t>10-5  Check the amount · pay by card</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="3" t="inlineStr">
+        <is>
+          <t>10-6  Check the payment · extra payment</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3213,6 +3612,42 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>An agency says it has no «A.i content payment» menu</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Check that they logged in with the agency ID. The menu appears only for agency accounts (not branch or HQ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>An agency sees «Head office has not opened A.i content payment yet»</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>It is not broken. It shows until HQ presses «Turn ON» for auto-billing in Finance › 🏢 AI Usage Fee (test period).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>An agency wants to remove a student they already paid for</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>It cannot be done on the agency screen. HQ handles refunds.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>